<commit_message>
just a regular update regarding DSA C-CPP
</commit_message>
<xml_diff>
--- a/Data Analytics/DataAnalytics All topics and pyq.xlsx
+++ b/Data Analytics/DataAnalytics All topics and pyq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\MCA-Sem2All\Data Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E16242-DEE6-4005-9FA5-0797199F0EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA319124-FEF8-41B9-9025-203F35072E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1400" yWindow="830" windowWidth="14400" windowHeight="9250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>unit 1</t>
   </si>
@@ -214,6 +214,56 @@
   </si>
   <si>
     <t>Spatial Data Analysis</t>
+  </si>
+  <si>
+    <t>Outliers</t>
+  </si>
+  <si>
+    <t>Lasso Regression</t>
+  </si>
+  <si>
+    <t>Steam processong</t>
+  </si>
+  <si>
+    <t>Data Processing</t>
+  </si>
+  <si>
+    <t>CLIQue clistering</t>
+  </si>
+  <si>
+    <t>diff . Supervised and unsupervised learning</t>
+  </si>
+  <si>
+    <t>Big Data , Small Data differences</t>
+  </si>
+  <si>
+    <t>Neural Netoworks</t>
+  </si>
+  <si>
+    <t>Artificial neural netwoks</t>
+  </si>
+  <si>
+    <t>union , intersection , complement, bold union , intersection on fuzzy sets
+give examples</t>
+  </si>
+  <si>
+    <t>flajolet martin alforithms</t>
+  </si>
+  <si>
+    <t>data stream filtering alforithm and processing</t>
+  </si>
+  <si>
+    <t>apriory algorithm , solve problem of 6 transactions , support 
+threshold =50% and confidence= 60% show strong association rules</t>
+  </si>
+  <si>
+    <t>what are the components of haddop</t>
+  </si>
+  <si>
+    <t>draw diagram of hadoop ecosystem</t>
+  </si>
+  <si>
+    <t>PYQ Paper 1</t>
   </si>
 </sst>
 </file>
@@ -249,8 +299,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A86"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.6328125" customWidth="1"/>
@@ -847,6 +900,86 @@
         <v>61</v>
       </c>
     </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A81" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>